<commit_message>
improve pitch detection (scales) to 99.49%
</commit_message>
<xml_diff>
--- a/src/tests/data/pitch_data/Shawn A Major Scale.xlsx
+++ b/src/tests/data/pitch_data/Shawn A Major Scale.xlsx
@@ -177,11 +177,11 @@
           <c:showPercent val="0"/>
           <c:showBubbleSize val="0"/>
         </c:dLbls>
-        <c:axId val="214941747"/>
-        <c:axId val="344573039"/>
+        <c:axId val="1615874089"/>
+        <c:axId val="402994849"/>
       </c:scatterChart>
       <c:valAx>
-        <c:axId val="214941747"/>
+        <c:axId val="1615874089"/>
         <c:scaling>
           <c:orientation val="minMax"/>
           <c:max val="32.448"/>
@@ -237,10 +237,10 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="344573039"/>
+        <c:crossAx val="402994849"/>
       </c:valAx>
       <c:valAx>
-        <c:axId val="344573039"/>
+        <c:axId val="402994849"/>
         <c:scaling>
           <c:orientation val="minMax"/>
           <c:max val="5000.000000000004"/>
@@ -305,7 +305,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="214941747"/>
+        <c:crossAx val="1615874089"/>
       </c:valAx>
     </c:plotArea>
     <c:plotVisOnly val="1"/>
@@ -19869,1698 +19869,862 @@
       </c>
     </row>
     <row r="2418" ht="15.75" customHeight="1">
-      <c r="A2418" s="2">
-        <v>30.01833333333333</v>
-      </c>
+      <c r="A2418" s="2"/>
     </row>
     <row r="2419" ht="15.75" customHeight="1">
-      <c r="A2419" s="2">
-        <v>30.02833333333334</v>
-      </c>
-      <c r="B2419" s="3">
-        <v>296.413818359375</v>
-      </c>
+      <c r="A2419" s="2"/>
+      <c r="B2419" s="3"/>
     </row>
     <row r="2420" ht="15.75" customHeight="1">
-      <c r="A2420" s="2">
-        <v>30.03833333333333</v>
-      </c>
-      <c r="B2420" s="3">
-        <v>313.689453125</v>
-      </c>
+      <c r="A2420" s="2"/>
+      <c r="B2420" s="3"/>
     </row>
     <row r="2421" ht="15.75" customHeight="1">
-      <c r="A2421" s="2">
-        <v>30.04833333333333</v>
-      </c>
-      <c r="B2421" s="3">
-        <v>313.502685546875</v>
-      </c>
+      <c r="A2421" s="2"/>
+      <c r="B2421" s="3"/>
     </row>
     <row r="2422" ht="15.75" customHeight="1">
-      <c r="A2422" s="2">
-        <v>30.05833333333333</v>
-      </c>
-      <c r="B2422" s="3">
-        <v>307.9426574707031</v>
-      </c>
+      <c r="A2422" s="2"/>
+      <c r="B2422" s="3"/>
     </row>
     <row r="2423" ht="15.75" customHeight="1">
-      <c r="A2423" s="2">
-        <v>30.06833333333334</v>
-      </c>
-      <c r="B2423" s="3">
-        <v>307.666259765625</v>
-      </c>
+      <c r="A2423" s="2"/>
+      <c r="B2423" s="3"/>
     </row>
     <row r="2424" ht="15.75" customHeight="1">
-      <c r="A2424" s="2">
-        <v>30.07833333333333</v>
-      </c>
-      <c r="B2424" s="3">
-        <v>302.1881103515625</v>
-      </c>
+      <c r="A2424" s="2"/>
+      <c r="B2424" s="3"/>
     </row>
     <row r="2425" ht="15.75" customHeight="1">
-      <c r="A2425" s="2">
-        <v>30.08833333333333</v>
-      </c>
-      <c r="B2425" s="3">
-        <v>296.5359191894531</v>
-      </c>
+      <c r="A2425" s="2"/>
+      <c r="B2425" s="3"/>
     </row>
     <row r="2426" ht="15.75" customHeight="1">
-      <c r="A2426" s="2">
-        <v>30.09833333333334</v>
-      </c>
-      <c r="B2426" s="3">
-        <v>280.7447509765625</v>
-      </c>
+      <c r="A2426" s="2"/>
+      <c r="B2426" s="3"/>
     </row>
     <row r="2427" ht="15.75" customHeight="1">
-      <c r="A2427" s="2">
-        <v>30.10833333333333</v>
-      </c>
-      <c r="B2427" s="3">
-        <v>275.8684387207031</v>
-      </c>
+      <c r="A2427" s="2"/>
+      <c r="B2427" s="3"/>
     </row>
     <row r="2428" ht="15.75" customHeight="1">
-      <c r="A2428" s="2">
-        <v>30.11833333333333</v>
-      </c>
-      <c r="B2428" s="3">
-        <v>271.3414001464844</v>
-      </c>
+      <c r="A2428" s="2"/>
+      <c r="B2428" s="3"/>
     </row>
     <row r="2429" ht="15.75" customHeight="1">
-      <c r="A2429" s="2">
-        <v>30.12833333333333</v>
-      </c>
-      <c r="B2429" s="3">
-        <v>275.2024841308594</v>
-      </c>
+      <c r="A2429" s="2"/>
+      <c r="B2429" s="3"/>
     </row>
     <row r="2430" ht="15.75" customHeight="1">
-      <c r="A2430" s="2">
-        <v>30.13833333333334</v>
-      </c>
-      <c r="B2430" s="3">
-        <v>275.6507568359375</v>
-      </c>
+      <c r="A2430" s="2"/>
+      <c r="B2430" s="3"/>
     </row>
     <row r="2431" ht="15.75" customHeight="1">
-      <c r="A2431" s="2">
-        <v>30.14833333333333</v>
-      </c>
-      <c r="B2431" s="3">
-        <v>275.5104064941406</v>
-      </c>
+      <c r="A2431" s="2"/>
+      <c r="B2431" s="3"/>
     </row>
     <row r="2432" ht="15.75" customHeight="1">
-      <c r="A2432" s="2">
-        <v>30.15833333333333</v>
-      </c>
-      <c r="B2432" s="3">
-        <v>274.6817016601562</v>
-      </c>
+      <c r="A2432" s="2"/>
+      <c r="B2432" s="3"/>
     </row>
     <row r="2433" ht="15.75" customHeight="1">
-      <c r="A2433" s="2">
-        <v>30.16833333333334</v>
-      </c>
-      <c r="B2433" s="3">
-        <v>271.5448303222656</v>
-      </c>
+      <c r="A2433" s="2"/>
+      <c r="B2433" s="3"/>
     </row>
     <row r="2434" ht="15.75" customHeight="1">
-      <c r="A2434" s="2">
-        <v>30.17833333333333</v>
-      </c>
-      <c r="B2434" s="3">
-        <v>267.0676879882812</v>
-      </c>
+      <c r="A2434" s="2"/>
+      <c r="B2434" s="3"/>
     </row>
     <row r="2435" ht="15.75" customHeight="1">
-      <c r="A2435" s="2">
-        <v>30.18833333333333</v>
-      </c>
-      <c r="B2435" s="3">
-        <v>258.7024230957031</v>
-      </c>
+      <c r="A2435" s="2"/>
+      <c r="B2435" s="3"/>
     </row>
     <row r="2436" ht="15.75" customHeight="1">
-      <c r="A2436" s="2">
-        <v>30.19833333333333</v>
-      </c>
-      <c r="B2436" s="3">
-        <v>228.4591674804688</v>
-      </c>
+      <c r="A2436" s="2"/>
+      <c r="B2436" s="3"/>
     </row>
     <row r="2437" ht="15.75" customHeight="1">
-      <c r="A2437" s="2">
-        <v>30.20833333333334</v>
-      </c>
-      <c r="B2437" s="3">
-        <v>225.8016967773438</v>
-      </c>
+      <c r="A2437" s="2"/>
+      <c r="B2437" s="3"/>
     </row>
     <row r="2438" ht="15.75" customHeight="1">
-      <c r="A2438" s="2">
-        <v>30.21833333333333</v>
-      </c>
-      <c r="B2438" s="3">
-        <v>225.6523284912109</v>
-      </c>
+      <c r="A2438" s="2"/>
+      <c r="B2438" s="3"/>
     </row>
     <row r="2439" ht="15.75" customHeight="1">
-      <c r="A2439" s="2">
-        <v>30.22833333333334</v>
-      </c>
-      <c r="B2439" s="3">
-        <v>225.5028076171875</v>
-      </c>
+      <c r="A2439" s="2"/>
+      <c r="B2439" s="3"/>
     </row>
     <row r="2440" ht="15.75" customHeight="1">
-      <c r="A2440" s="2">
-        <v>30.22833333333334</v>
-      </c>
+      <c r="A2440" s="2"/>
     </row>
     <row r="2441" ht="15.75" customHeight="1">
-      <c r="A2441" s="2">
-        <v>30.23833333333334</v>
-      </c>
-      <c r="B2441" s="3">
-        <v>66.66526794433594</v>
-      </c>
+      <c r="A2441" s="2"/>
+      <c r="B2441" s="3"/>
     </row>
     <row r="2442" ht="15.75" customHeight="1">
-      <c r="A2442" s="2">
-        <v>30.24833333333333</v>
-      </c>
-      <c r="B2442" s="3">
-        <v>67.21562194824219</v>
-      </c>
+      <c r="A2442" s="2"/>
+      <c r="B2442" s="3"/>
     </row>
     <row r="2443" ht="15.75" customHeight="1">
-      <c r="A2443" s="2">
-        <v>30.24833333333333</v>
-      </c>
+      <c r="A2443" s="2"/>
     </row>
     <row r="2444" ht="15.75" customHeight="1">
-      <c r="A2444" s="2">
-        <v>30.25833333333333</v>
-      </c>
-      <c r="B2444" s="3">
-        <v>210.5656280517578</v>
-      </c>
+      <c r="A2444" s="2"/>
+      <c r="B2444" s="3"/>
     </row>
     <row r="2445" ht="15.75" customHeight="1">
-      <c r="A2445" s="2">
-        <v>30.26833333333333</v>
-      </c>
-      <c r="B2445" s="3">
-        <v>205.1702728271484</v>
-      </c>
+      <c r="A2445" s="2"/>
+      <c r="B2445" s="3"/>
     </row>
     <row r="2446" ht="15.75" customHeight="1">
-      <c r="A2446" s="2">
-        <v>30.27833333333334</v>
-      </c>
-      <c r="B2446" s="3">
-        <v>216.2235870361328</v>
-      </c>
+      <c r="A2446" s="2"/>
+      <c r="B2446" s="3"/>
     </row>
     <row r="2447" ht="15.75" customHeight="1">
-      <c r="A2447" s="2">
-        <v>30.28833333333333</v>
-      </c>
-      <c r="B2447" s="3">
-        <v>216.2536315917969</v>
-      </c>
+      <c r="A2447" s="2"/>
+      <c r="B2447" s="3"/>
     </row>
     <row r="2448" ht="15.75" customHeight="1">
-      <c r="A2448" s="2">
-        <v>30.29833333333333</v>
-      </c>
-      <c r="B2448" s="3">
-        <v>222.1985321044922</v>
-      </c>
+      <c r="A2448" s="2"/>
+      <c r="B2448" s="3"/>
     </row>
     <row r="2449" ht="15.75" customHeight="1">
-      <c r="A2449" s="2">
-        <v>30.39833333333333</v>
-      </c>
+      <c r="A2449" s="2"/>
     </row>
     <row r="2450" ht="15.75" customHeight="1">
-      <c r="A2450" s="2">
-        <v>30.40833333333333</v>
-      </c>
-      <c r="B2450" s="3">
-        <v>190.3849639892578</v>
-      </c>
+      <c r="A2450" s="2"/>
+      <c r="B2450" s="3"/>
     </row>
     <row r="2451" ht="15.75" customHeight="1">
-      <c r="A2451" s="2">
-        <v>30.41833333333334</v>
-      </c>
-      <c r="B2451" s="3">
-        <v>186.1109619140625</v>
-      </c>
+      <c r="A2451" s="2"/>
+      <c r="B2451" s="3"/>
     </row>
     <row r="2452" ht="15.75" customHeight="1">
-      <c r="A2452" s="2">
-        <v>30.42833333333333</v>
-      </c>
-      <c r="B2452" s="3">
-        <v>185.8955993652344</v>
-      </c>
+      <c r="A2452" s="2"/>
+      <c r="B2452" s="3"/>
     </row>
     <row r="2453" ht="15.75" customHeight="1">
-      <c r="A2453" s="2">
-        <v>30.43833333333333</v>
-      </c>
-      <c r="B2453" s="3">
-        <v>183.8423614501953</v>
-      </c>
+      <c r="A2453" s="2"/>
+      <c r="B2453" s="3"/>
     </row>
     <row r="2454" ht="15.75" customHeight="1">
-      <c r="A2454" s="2">
-        <v>30.44833333333333</v>
-      </c>
-      <c r="B2454" s="3">
-        <v>181.9223327636719</v>
-      </c>
+      <c r="A2454" s="2"/>
+      <c r="B2454" s="3"/>
     </row>
     <row r="2455" ht="15.75" customHeight="1">
-      <c r="A2455" s="2">
-        <v>30.45833333333334</v>
-      </c>
-      <c r="B2455" s="3">
-        <v>179.6249237060547</v>
-      </c>
+      <c r="A2455" s="2"/>
+      <c r="B2455" s="3"/>
     </row>
     <row r="2456" ht="15.75" customHeight="1">
-      <c r="A2456" s="2">
-        <v>30.46833333333333</v>
-      </c>
-      <c r="B2456" s="3">
-        <v>173.9088897705078</v>
-      </c>
+      <c r="A2456" s="2"/>
+      <c r="B2456" s="3"/>
     </row>
     <row r="2457" ht="15.75" customHeight="1">
-      <c r="A2457" s="2">
-        <v>30.47833333333334</v>
-      </c>
-      <c r="B2457" s="3">
-        <v>172.0510711669922</v>
-      </c>
+      <c r="A2457" s="2"/>
+      <c r="B2457" s="3"/>
     </row>
     <row r="2458" ht="15.75" customHeight="1">
-      <c r="A2458" s="2">
-        <v>30.48833333333334</v>
-      </c>
-      <c r="B2458" s="3">
-        <v>173.8451995849609</v>
-      </c>
+      <c r="A2458" s="2"/>
+      <c r="B2458" s="3"/>
     </row>
     <row r="2459" ht="15.75" customHeight="1">
-      <c r="A2459" s="2">
-        <v>30.49833333333333</v>
-      </c>
-      <c r="B2459" s="3">
-        <v>173.9820556640625</v>
-      </c>
+      <c r="A2459" s="2"/>
+      <c r="B2459" s="3"/>
     </row>
     <row r="2460" ht="15.75" customHeight="1">
-      <c r="A2460" s="2">
-        <v>30.50833333333333</v>
-      </c>
-      <c r="B2460" s="3">
-        <v>177.7795257568359</v>
-      </c>
+      <c r="A2460" s="2"/>
+      <c r="B2460" s="3"/>
     </row>
     <row r="2461" ht="15.75" customHeight="1">
-      <c r="A2461" s="2">
-        <v>30.51833333333333</v>
-      </c>
-      <c r="B2461" s="3">
-        <v>275.8204650878906</v>
-      </c>
+      <c r="A2461" s="2"/>
+      <c r="B2461" s="3"/>
     </row>
     <row r="2462" ht="15.75" customHeight="1">
-      <c r="A2462" s="2">
-        <v>30.52833333333334</v>
-      </c>
-      <c r="B2462" s="3">
-        <v>275.81982421875</v>
-      </c>
+      <c r="A2462" s="2"/>
+      <c r="B2462" s="3"/>
     </row>
     <row r="2463" ht="15.75" customHeight="1">
-      <c r="A2463" s="2">
-        <v>30.53833333333333</v>
-      </c>
-      <c r="B2463" s="3">
-        <v>177.7364654541016</v>
-      </c>
+      <c r="A2463" s="2"/>
+      <c r="B2463" s="3"/>
     </row>
     <row r="2464" ht="15.75" customHeight="1">
-      <c r="A2464" s="2">
-        <v>30.64833333333333</v>
-      </c>
+      <c r="A2464" s="2"/>
     </row>
     <row r="2465" ht="15.75" customHeight="1">
-      <c r="A2465" s="2">
-        <v>30.65833333333333</v>
-      </c>
-      <c r="B2465" s="3">
-        <v>170.2234039306641</v>
-      </c>
+      <c r="A2465" s="2"/>
+      <c r="B2465" s="3"/>
     </row>
     <row r="2466" ht="15.75" customHeight="1">
-      <c r="A2466" s="2">
-        <v>30.66833333333334</v>
-      </c>
-      <c r="B2466" s="3">
-        <v>140.3311004638672</v>
-      </c>
+      <c r="A2466" s="2"/>
+      <c r="B2466" s="3"/>
     </row>
     <row r="2467" ht="15.75" customHeight="1">
-      <c r="A2467" s="2">
-        <v>30.67833333333333</v>
-      </c>
-      <c r="B2467" s="3">
-        <v>139.1581878662109</v>
-      </c>
+      <c r="A2467" s="2"/>
+      <c r="B2467" s="3"/>
     </row>
     <row r="2468" ht="15.75" customHeight="1">
-      <c r="A2468" s="2">
-        <v>30.68833333333333</v>
-      </c>
-      <c r="B2468" s="3">
-        <v>140.3692016601562</v>
-      </c>
+      <c r="A2468" s="2"/>
+      <c r="B2468" s="3"/>
     </row>
     <row r="2469" ht="15.75" customHeight="1">
-      <c r="A2469" s="2">
-        <v>30.69833333333333</v>
-      </c>
-      <c r="B2469" s="3">
-        <v>141.5605773925781</v>
-      </c>
+      <c r="A2469" s="2"/>
+      <c r="B2469" s="3"/>
     </row>
     <row r="2470" ht="15.75" customHeight="1">
-      <c r="A2470" s="2">
-        <v>30.70833333333334</v>
-      </c>
-      <c r="B2470" s="3">
-        <v>142.8651428222656</v>
-      </c>
+      <c r="A2470" s="2"/>
+      <c r="B2470" s="3"/>
     </row>
     <row r="2471" ht="15.75" customHeight="1">
-      <c r="A2471" s="2">
-        <v>30.71833333333333</v>
-      </c>
-      <c r="B2471" s="3">
-        <v>142.9144287109375</v>
-      </c>
+      <c r="A2471" s="2"/>
+      <c r="B2471" s="3"/>
     </row>
     <row r="2472" ht="15.75" customHeight="1">
-      <c r="A2472" s="2">
-        <v>30.72833333333334</v>
-      </c>
-      <c r="B2472" s="3">
-        <v>144.1475372314453</v>
-      </c>
+      <c r="A2472" s="2"/>
+      <c r="B2472" s="3"/>
     </row>
     <row r="2473" ht="15.75" customHeight="1">
-      <c r="A2473" s="2">
-        <v>30.73833333333334</v>
-      </c>
-      <c r="B2473" s="3">
-        <v>142.8850555419922</v>
-      </c>
+      <c r="A2473" s="2"/>
+      <c r="B2473" s="3"/>
     </row>
     <row r="2474" ht="15.75" customHeight="1">
-      <c r="A2474" s="2">
-        <v>30.74833333333333</v>
-      </c>
-      <c r="B2474" s="3">
-        <v>142.7484893798828</v>
-      </c>
+      <c r="A2474" s="2"/>
+      <c r="B2474" s="3"/>
     </row>
     <row r="2475" ht="15.75" customHeight="1">
-      <c r="A2475" s="2">
-        <v>30.75833333333333</v>
-      </c>
-      <c r="B2475" s="3">
-        <v>140.3112030029297</v>
-      </c>
+      <c r="A2475" s="2"/>
+      <c r="B2475" s="3"/>
     </row>
     <row r="2476" ht="15.75" customHeight="1">
-      <c r="A2476" s="2">
-        <v>30.76833333333333</v>
-      </c>
-      <c r="B2476" s="3">
-        <v>96.40227508544922</v>
-      </c>
+      <c r="A2476" s="2"/>
+      <c r="B2476" s="3"/>
     </row>
     <row r="2477" ht="15.75" customHeight="1">
-      <c r="A2477" s="2">
-        <v>30.77833333333334</v>
-      </c>
-      <c r="B2477" s="3">
-        <v>97.5615234375</v>
-      </c>
+      <c r="A2477" s="2"/>
+      <c r="B2477" s="3"/>
     </row>
     <row r="2478" ht="15.75" customHeight="1">
-      <c r="A2478" s="2">
-        <v>30.78833333333333</v>
-      </c>
-      <c r="B2478" s="3">
-        <v>135.5334777832031</v>
-      </c>
+      <c r="A2478" s="2"/>
+      <c r="B2478" s="3"/>
     </row>
     <row r="2479" ht="15.75" customHeight="1">
-      <c r="A2479" s="2">
-        <v>30.79833333333333</v>
-      </c>
-      <c r="B2479" s="3">
-        <v>139.0970916748047</v>
-      </c>
+      <c r="A2479" s="2"/>
+      <c r="B2479" s="3"/>
     </row>
     <row r="2480" ht="15.75" customHeight="1">
-      <c r="A2480" s="2">
-        <v>30.80833333333333</v>
-      </c>
-      <c r="B2480" s="3">
-        <v>137.9429168701172</v>
-      </c>
+      <c r="A2480" s="2"/>
+      <c r="B2480" s="3"/>
     </row>
     <row r="2481" ht="15.75" customHeight="1">
-      <c r="A2481" s="2">
-        <v>30.81833333333334</v>
-      </c>
-      <c r="B2481" s="3">
-        <v>140.3161468505859</v>
-      </c>
+      <c r="A2481" s="2"/>
+      <c r="B2481" s="3"/>
     </row>
     <row r="2482" ht="15.75" customHeight="1">
-      <c r="A2482" s="2">
-        <v>30.82833333333333</v>
-      </c>
-      <c r="B2482" s="3">
-        <v>137.9392852783203</v>
-      </c>
+      <c r="A2482" s="2"/>
+      <c r="B2482" s="3"/>
     </row>
     <row r="2483" ht="15.75" customHeight="1">
-      <c r="A2483" s="2">
-        <v>30.83833333333333</v>
-      </c>
-      <c r="B2483" s="3">
-        <v>137.8979797363281</v>
-      </c>
+      <c r="A2483" s="2"/>
+      <c r="B2483" s="3"/>
     </row>
     <row r="2484" ht="15.75" customHeight="1">
-      <c r="A2484" s="2">
-        <v>30.84833333333334</v>
-      </c>
-      <c r="B2484" s="3">
-        <v>135.6597900390625</v>
-      </c>
+      <c r="A2484" s="2"/>
+      <c r="B2484" s="3"/>
     </row>
     <row r="2485" ht="15.75" customHeight="1">
-      <c r="A2485" s="2">
-        <v>30.85833333333333</v>
-      </c>
-      <c r="B2485" s="3">
-        <v>136.7790985107422</v>
-      </c>
+      <c r="A2485" s="2"/>
+      <c r="B2485" s="3"/>
     </row>
     <row r="2486" ht="15.75" customHeight="1">
-      <c r="A2486" s="2">
-        <v>30.86833333333333</v>
-      </c>
-      <c r="B2486" s="3">
-        <v>136.8139190673828</v>
-      </c>
+      <c r="A2486" s="2"/>
+      <c r="B2486" s="3"/>
     </row>
     <row r="2487" ht="15.75" customHeight="1">
-      <c r="A2487" s="2">
-        <v>30.87833333333333</v>
-      </c>
-      <c r="B2487" s="3">
-        <v>136.7608947753906</v>
-      </c>
+      <c r="A2487" s="2"/>
+      <c r="B2487" s="3"/>
     </row>
     <row r="2488" ht="15.75" customHeight="1">
-      <c r="A2488" s="2">
-        <v>30.87833333333333</v>
-      </c>
+      <c r="A2488" s="2"/>
     </row>
     <row r="2489" ht="15.75" customHeight="1">
-      <c r="A2489" s="2">
-        <v>30.88833333333334</v>
-      </c>
-      <c r="B2489" s="3">
-        <v>666.6592407226562</v>
-      </c>
+      <c r="A2489" s="2"/>
+      <c r="B2489" s="3"/>
     </row>
     <row r="2490" ht="15.75" customHeight="1">
-      <c r="A2490" s="2">
-        <v>30.89833333333333</v>
-      </c>
-      <c r="B2490" s="3">
-        <v>668.4526977539062</v>
-      </c>
+      <c r="A2490" s="2"/>
+      <c r="B2490" s="3"/>
     </row>
     <row r="2491" ht="15.75" customHeight="1">
-      <c r="A2491" s="2">
-        <v>30.90833333333333</v>
-      </c>
-      <c r="B2491" s="3">
-        <v>668.676025390625</v>
-      </c>
+      <c r="A2491" s="2"/>
+      <c r="B2491" s="3"/>
     </row>
     <row r="2492" ht="15.75" customHeight="1">
-      <c r="A2492" s="2">
-        <v>30.90833333333333</v>
-      </c>
+      <c r="A2492" s="2"/>
     </row>
     <row r="2493" ht="15.75" customHeight="1">
-      <c r="A2493" s="2">
-        <v>30.91833333333334</v>
-      </c>
-      <c r="B2493" s="3">
-        <v>129.0462646484375</v>
-      </c>
+      <c r="A2493" s="2"/>
+      <c r="B2493" s="3"/>
     </row>
     <row r="2494" ht="15.75" customHeight="1">
-      <c r="A2494" s="2">
-        <v>30.92833333333333</v>
-      </c>
-      <c r="B2494" s="3">
-        <v>128.0414581298828</v>
-      </c>
+      <c r="A2494" s="2"/>
+      <c r="B2494" s="3"/>
     </row>
     <row r="2495" ht="15.75" customHeight="1">
-      <c r="A2495" s="2">
-        <v>30.93833333333333</v>
-      </c>
-      <c r="B2495" s="3">
-        <v>128.956787109375</v>
-      </c>
+      <c r="A2495" s="2"/>
+      <c r="B2495" s="3"/>
     </row>
     <row r="2496" ht="15.75" customHeight="1">
-      <c r="A2496" s="2">
-        <v>30.94833333333333</v>
-      </c>
-      <c r="B2496" s="3">
-        <v>128.9646148681641</v>
-      </c>
+      <c r="A2496" s="2"/>
+      <c r="B2496" s="3"/>
     </row>
     <row r="2497" ht="15.75" customHeight="1">
-      <c r="A2497" s="2">
-        <v>30.95833333333334</v>
-      </c>
-      <c r="B2497" s="3">
-        <v>129.0768890380859</v>
-      </c>
+      <c r="A2497" s="2"/>
+      <c r="B2497" s="3"/>
     </row>
     <row r="2498" ht="15.75" customHeight="1">
-      <c r="A2498" s="2">
-        <v>30.96833333333333</v>
-      </c>
-      <c r="B2498" s="3">
-        <v>131.1800079345703</v>
-      </c>
+      <c r="A2498" s="2"/>
+      <c r="B2498" s="3"/>
     </row>
     <row r="2499" ht="15.75" customHeight="1">
-      <c r="A2499" s="2">
-        <v>30.97833333333334</v>
-      </c>
-      <c r="B2499" s="3">
-        <v>133.3024597167969</v>
-      </c>
+      <c r="A2499" s="2"/>
+      <c r="B2499" s="3"/>
     </row>
     <row r="2500" ht="15.75" customHeight="1">
-      <c r="A2500" s="2">
-        <v>30.98833333333334</v>
-      </c>
-      <c r="B2500" s="3">
-        <v>134.4378356933594</v>
-      </c>
+      <c r="A2500" s="2"/>
+      <c r="B2500" s="3"/>
     </row>
     <row r="2501" ht="15.75" customHeight="1">
-      <c r="A2501" s="2">
-        <v>30.99833333333333</v>
-      </c>
-      <c r="B2501" s="3">
-        <v>135.5171813964844</v>
-      </c>
+      <c r="A2501" s="2"/>
+      <c r="B2501" s="3"/>
     </row>
     <row r="2502" ht="15.75" customHeight="1">
-      <c r="A2502" s="2">
-        <v>31.00833333333333</v>
-      </c>
-      <c r="B2502" s="3">
-        <v>135.5433044433594</v>
-      </c>
+      <c r="A2502" s="2"/>
+      <c r="B2502" s="3"/>
     </row>
     <row r="2503" ht="15.75" customHeight="1">
-      <c r="A2503" s="2">
-        <v>31.01833333333333</v>
-      </c>
-      <c r="B2503" s="3">
-        <v>135.6137390136719</v>
-      </c>
+      <c r="A2503" s="2"/>
+      <c r="B2503" s="3"/>
     </row>
     <row r="2504" ht="15.75" customHeight="1">
-      <c r="A2504" s="2">
-        <v>31.02833333333334</v>
-      </c>
-      <c r="B2504" s="3">
-        <v>133.3402404785156</v>
-      </c>
+      <c r="A2504" s="2"/>
+      <c r="B2504" s="3"/>
     </row>
     <row r="2505" ht="15.75" customHeight="1">
-      <c r="A2505" s="2">
-        <v>31.03833333333333</v>
-      </c>
-      <c r="B2505" s="3">
-        <v>133.3137664794922</v>
-      </c>
+      <c r="A2505" s="2"/>
+      <c r="B2505" s="3"/>
     </row>
     <row r="2506" ht="15.75" customHeight="1">
-      <c r="A2506" s="2">
-        <v>31.04833333333333</v>
-      </c>
-      <c r="B2506" s="3">
-        <v>133.2602996826172</v>
-      </c>
+      <c r="A2506" s="2"/>
+      <c r="B2506" s="3"/>
     </row>
     <row r="2507" ht="15.75" customHeight="1">
-      <c r="A2507" s="2">
-        <v>31.05833333333333</v>
-      </c>
-      <c r="B2507" s="3">
-        <v>134.5690002441406</v>
-      </c>
+      <c r="A2507" s="2"/>
+      <c r="B2507" s="3"/>
     </row>
     <row r="2508" ht="15.75" customHeight="1">
-      <c r="A2508" s="2">
-        <v>31.06833333333334</v>
-      </c>
-      <c r="B2508" s="3">
-        <v>134.4018249511719</v>
-      </c>
+      <c r="A2508" s="2"/>
+      <c r="B2508" s="3"/>
     </row>
     <row r="2509" ht="15.75" customHeight="1">
-      <c r="A2509" s="2">
-        <v>31.07833333333333</v>
-      </c>
+      <c r="A2509" s="2"/>
     </row>
     <row r="2510" ht="15.75" customHeight="1">
-      <c r="A2510" s="2">
-        <v>31.08833333333333</v>
-      </c>
-      <c r="B2510" s="3">
-        <v>131.3175048828125</v>
-      </c>
+      <c r="A2510" s="2"/>
+      <c r="B2510" s="3"/>
     </row>
     <row r="2511" ht="15.75" customHeight="1">
-      <c r="A2511" s="2">
-        <v>31.09833333333334</v>
-      </c>
-      <c r="B2511" s="3">
-        <v>131.3292999267578</v>
-      </c>
+      <c r="A2511" s="2"/>
+      <c r="B2511" s="3"/>
     </row>
     <row r="2512" ht="15.75" customHeight="1">
-      <c r="A2512" s="2">
-        <v>31.10833333333333</v>
-      </c>
-      <c r="B2512" s="3">
-        <v>134.1376495361328</v>
-      </c>
+      <c r="A2512" s="2"/>
+      <c r="B2512" s="3"/>
     </row>
     <row r="2513" ht="15.75" customHeight="1">
-      <c r="A2513" s="2">
-        <v>31.11833333333333</v>
-      </c>
-      <c r="B2513" s="3">
-        <v>138.7544860839844</v>
-      </c>
+      <c r="A2513" s="2"/>
+      <c r="B2513" s="3"/>
     </row>
     <row r="2514" ht="15.75" customHeight="1">
-      <c r="A2514" s="2">
-        <v>31.13833333333334</v>
-      </c>
+      <c r="A2514" s="2"/>
     </row>
     <row r="2515" ht="15.75" customHeight="1">
-      <c r="A2515" s="2">
-        <v>31.14833333333333</v>
-      </c>
-      <c r="B2515" s="3">
-        <v>75.0950927734375</v>
-      </c>
+      <c r="A2515" s="2"/>
+      <c r="B2515" s="3"/>
     </row>
     <row r="2516" ht="15.75" customHeight="1">
-      <c r="A2516" s="2">
-        <v>31.15833333333333</v>
-      </c>
-      <c r="B2516" s="3">
-        <v>75.10176849365234</v>
-      </c>
+      <c r="A2516" s="2"/>
+      <c r="B2516" s="3"/>
     </row>
     <row r="2517" ht="15.75" customHeight="1">
-      <c r="A2517" s="2">
-        <v>31.15833333333333</v>
-      </c>
+      <c r="A2517" s="2"/>
     </row>
     <row r="2518" ht="15.75" customHeight="1">
-      <c r="A2518" s="2">
-        <v>31.16833333333334</v>
-      </c>
-      <c r="B2518" s="3">
-        <v>142.7483978271484</v>
-      </c>
+      <c r="A2518" s="2"/>
+      <c r="B2518" s="3"/>
     </row>
     <row r="2519" ht="15.75" customHeight="1">
-      <c r="A2519" s="2">
-        <v>31.17833333333333</v>
-      </c>
-      <c r="B2519" s="3">
-        <v>145.4806671142578</v>
-      </c>
+      <c r="A2519" s="2"/>
+      <c r="B2519" s="3"/>
     </row>
     <row r="2520" ht="15.75" customHeight="1">
-      <c r="A2520" s="2">
-        <v>31.18833333333333</v>
-      </c>
-      <c r="B2520" s="3">
-        <v>149.4460906982422</v>
-      </c>
+      <c r="A2520" s="2"/>
+      <c r="B2520" s="3"/>
     </row>
     <row r="2521" ht="15.75" customHeight="1">
-      <c r="A2521" s="2">
-        <v>31.19833333333333</v>
-      </c>
-      <c r="B2521" s="3">
-        <v>149.4608459472656</v>
-      </c>
+      <c r="A2521" s="2"/>
+      <c r="B2521" s="3"/>
     </row>
     <row r="2522" ht="15.75" customHeight="1">
-      <c r="A2522" s="2">
-        <v>31.20833333333334</v>
-      </c>
-      <c r="B2522" s="3">
-        <v>153.8675994873047</v>
-      </c>
+      <c r="A2522" s="2"/>
+      <c r="B2522" s="3"/>
     </row>
     <row r="2523" ht="15.75" customHeight="1">
-      <c r="A2523" s="2">
-        <v>31.21833333333333</v>
-      </c>
-      <c r="B2523" s="3">
-        <v>156.8602447509766</v>
-      </c>
+      <c r="A2523" s="2"/>
+      <c r="B2523" s="3"/>
     </row>
     <row r="2524" ht="15.75" customHeight="1">
-      <c r="A2524" s="2">
-        <v>31.22833333333334</v>
-      </c>
+      <c r="A2524" s="2"/>
     </row>
     <row r="2525" ht="15.75" customHeight="1">
-      <c r="A2525" s="2">
-        <v>31.23833333333334</v>
-      </c>
-      <c r="B2525" s="3">
-        <v>75.47272491455078</v>
-      </c>
+      <c r="A2525" s="2"/>
+      <c r="B2525" s="3"/>
     </row>
     <row r="2526" ht="15.75" customHeight="1">
-      <c r="A2526" s="2">
-        <v>31.24833333333333</v>
-      </c>
-      <c r="B2526" s="3">
-        <v>75.48187255859375</v>
-      </c>
+      <c r="A2526" s="2"/>
+      <c r="B2526" s="3"/>
     </row>
     <row r="2527" ht="15.75" customHeight="1">
-      <c r="A2527" s="2">
-        <v>31.25833333333333</v>
-      </c>
-      <c r="B2527" s="3">
-        <v>74.0745620727539</v>
-      </c>
+      <c r="A2527" s="2"/>
+      <c r="B2527" s="3"/>
     </row>
     <row r="2528" ht="15.75" customHeight="1">
-      <c r="A2528" s="2">
-        <v>31.26833333333333</v>
-      </c>
-      <c r="B2528" s="3">
-        <v>73.38856506347656</v>
-      </c>
+      <c r="A2528" s="2"/>
+      <c r="B2528" s="3"/>
     </row>
     <row r="2529" ht="15.75" customHeight="1">
-      <c r="A2529" s="2">
-        <v>31.27833333333334</v>
-      </c>
-      <c r="B2529" s="3">
-        <v>74.75662231445312</v>
-      </c>
+      <c r="A2529" s="2"/>
+      <c r="B2529" s="3"/>
     </row>
     <row r="2530" ht="15.75" customHeight="1">
-      <c r="A2530" s="2">
-        <v>31.28833333333333</v>
-      </c>
-      <c r="B2530" s="3">
-        <v>75.46623229980469</v>
-      </c>
+      <c r="A2530" s="2"/>
+      <c r="B2530" s="3"/>
     </row>
     <row r="2531" ht="15.75" customHeight="1">
-      <c r="A2531" s="2">
-        <v>31.29833333333333</v>
-      </c>
-      <c r="B2531" s="3">
-        <v>74.76567840576172</v>
-      </c>
+      <c r="A2531" s="2"/>
+      <c r="B2531" s="3"/>
     </row>
     <row r="2532" ht="15.75" customHeight="1">
-      <c r="A2532" s="2">
-        <v>31.29833333333333</v>
-      </c>
+      <c r="A2532" s="2"/>
     </row>
     <row r="2533" ht="15.75" customHeight="1">
-      <c r="A2533" s="2">
-        <v>31.30833333333333</v>
-      </c>
-      <c r="B2533" s="3">
-        <v>142.8518981933594</v>
-      </c>
+      <c r="A2533" s="2"/>
+      <c r="B2533" s="3"/>
     </row>
     <row r="2534" ht="15.75" customHeight="1">
-      <c r="A2534" s="2">
-        <v>31.31833333333334</v>
-      </c>
-      <c r="B2534" s="3">
-        <v>145.4219512939453</v>
-      </c>
+      <c r="A2534" s="2"/>
+      <c r="B2534" s="3"/>
     </row>
     <row r="2535" ht="15.75" customHeight="1">
-      <c r="A2535" s="2">
-        <v>31.32833333333333</v>
-      </c>
-      <c r="B2535" s="3">
-        <v>145.4058074951172</v>
-      </c>
+      <c r="A2535" s="2"/>
+      <c r="B2535" s="3"/>
     </row>
     <row r="2536" ht="15.75" customHeight="1">
-      <c r="A2536" s="2">
-        <v>31.33833333333333</v>
-      </c>
-      <c r="B2536" s="3">
-        <v>145.4136352539062</v>
-      </c>
+      <c r="A2536" s="2"/>
+      <c r="B2536" s="3"/>
     </row>
     <row r="2537" ht="15.75" customHeight="1">
-      <c r="A2537" s="2">
-        <v>31.34833333333334</v>
-      </c>
-      <c r="B2537" s="3">
-        <v>145.5023040771484</v>
-      </c>
+      <c r="A2537" s="2"/>
+      <c r="B2537" s="3"/>
     </row>
     <row r="2538" ht="15.75" customHeight="1">
-      <c r="A2538" s="2">
-        <v>31.35833333333333</v>
-      </c>
-      <c r="B2538" s="3">
-        <v>145.5411987304688</v>
-      </c>
+      <c r="A2538" s="2"/>
+      <c r="B2538" s="3"/>
     </row>
     <row r="2539" ht="15.75" customHeight="1">
-      <c r="A2539" s="2">
-        <v>31.36833333333333</v>
-      </c>
-      <c r="B2539" s="3">
-        <v>145.3330383300781</v>
-      </c>
+      <c r="A2539" s="2"/>
+      <c r="B2539" s="3"/>
     </row>
     <row r="2540" ht="15.75" customHeight="1">
-      <c r="A2540" s="2">
-        <v>31.37833333333333</v>
-      </c>
-      <c r="B2540" s="3">
-        <v>145.3914184570312</v>
-      </c>
+      <c r="A2540" s="2"/>
+      <c r="B2540" s="3"/>
     </row>
     <row r="2541" ht="15.75" customHeight="1">
-      <c r="A2541" s="2">
-        <v>31.38833333333334</v>
-      </c>
+      <c r="A2541" s="2"/>
     </row>
     <row r="2542" ht="15.75" customHeight="1">
-      <c r="A2542" s="2">
-        <v>31.39833333333333</v>
-      </c>
-      <c r="B2542" s="3">
-        <v>398.8481140136719</v>
-      </c>
+      <c r="A2542" s="2"/>
+      <c r="B2542" s="3"/>
     </row>
     <row r="2543" ht="15.75" customHeight="1">
-      <c r="A2543" s="2">
-        <v>31.40833333333333</v>
-      </c>
-      <c r="B2543" s="3">
-        <v>403.0940246582031</v>
-      </c>
+      <c r="A2543" s="2"/>
+      <c r="B2543" s="3"/>
     </row>
     <row r="2544" ht="15.75" customHeight="1">
-      <c r="A2544" s="2">
-        <v>31.41833333333334</v>
-      </c>
-      <c r="B2544" s="3">
-        <v>406.8507080078125</v>
-      </c>
+      <c r="A2544" s="2"/>
+      <c r="B2544" s="3"/>
     </row>
     <row r="2545" ht="15.75" customHeight="1">
-      <c r="A2545" s="2">
-        <v>31.42833333333333</v>
-      </c>
-      <c r="B2545" s="3">
-        <v>408.7770385742188</v>
-      </c>
+      <c r="A2545" s="2"/>
+      <c r="B2545" s="3"/>
     </row>
     <row r="2546" ht="15.75" customHeight="1">
-      <c r="A2546" s="2">
-        <v>31.43833333333333</v>
-      </c>
-      <c r="B2546" s="3">
-        <v>409.3056030273438</v>
-      </c>
+      <c r="A2546" s="2"/>
+      <c r="B2546" s="3"/>
     </row>
     <row r="2547" ht="15.75" customHeight="1">
-      <c r="A2547" s="2">
-        <v>31.44833333333333</v>
-      </c>
-      <c r="B2547" s="3">
-        <v>408.4354248046875</v>
-      </c>
+      <c r="A2547" s="2"/>
+      <c r="B2547" s="3"/>
     </row>
     <row r="2548" ht="15.75" customHeight="1">
-      <c r="A2548" s="2">
-        <v>31.45833333333334</v>
-      </c>
-      <c r="B2548" s="3">
-        <v>406.2526245117188</v>
-      </c>
+      <c r="A2548" s="2"/>
+      <c r="B2548" s="3"/>
     </row>
     <row r="2549" ht="15.75" customHeight="1">
-      <c r="A2549" s="2">
-        <v>31.46833333333333</v>
-      </c>
-      <c r="B2549" s="3">
-        <v>402.1426391601562</v>
-      </c>
+      <c r="A2549" s="2"/>
+      <c r="B2549" s="3"/>
     </row>
     <row r="2550" ht="15.75" customHeight="1">
-      <c r="A2550" s="2">
-        <v>31.47833333333334</v>
-      </c>
-      <c r="B2550" s="3">
-        <v>398.0650939941406</v>
-      </c>
+      <c r="A2550" s="2"/>
+      <c r="B2550" s="3"/>
     </row>
     <row r="2551" ht="15.75" customHeight="1">
-      <c r="A2551" s="2">
-        <v>31.48833333333334</v>
-      </c>
-      <c r="B2551" s="3">
-        <v>394.5170593261719</v>
-      </c>
+      <c r="A2551" s="2"/>
+      <c r="B2551" s="3"/>
     </row>
     <row r="2552" ht="15.75" customHeight="1">
-      <c r="A2552" s="2">
-        <v>31.49833333333333</v>
-      </c>
-      <c r="B2552" s="3">
-        <v>391.7158203125</v>
-      </c>
+      <c r="A2552" s="2"/>
+      <c r="B2552" s="3"/>
     </row>
     <row r="2553" ht="15.75" customHeight="1">
-      <c r="A2553" s="2">
-        <v>31.50833333333333</v>
-      </c>
-      <c r="B2553" s="3">
-        <v>388.7644653320312</v>
-      </c>
+      <c r="A2553" s="2"/>
+      <c r="B2553" s="3"/>
     </row>
     <row r="2554" ht="15.75" customHeight="1">
-      <c r="A2554" s="2">
-        <v>31.51833333333333</v>
-      </c>
-      <c r="B2554" s="3">
-        <v>385.0213317871094</v>
-      </c>
+      <c r="A2554" s="2"/>
+      <c r="B2554" s="3"/>
     </row>
     <row r="2555" ht="15.75" customHeight="1">
-      <c r="A2555" s="2">
-        <v>31.52833333333334</v>
-      </c>
-      <c r="B2555" s="3">
-        <v>381.6622924804688</v>
-      </c>
+      <c r="A2555" s="2"/>
+      <c r="B2555" s="3"/>
     </row>
     <row r="2556" ht="15.75" customHeight="1">
-      <c r="A2556" s="2">
-        <v>31.53833333333333</v>
-      </c>
-      <c r="B2556" s="3">
-        <v>378.7737426757812</v>
-      </c>
+      <c r="A2556" s="2"/>
+      <c r="B2556" s="3"/>
     </row>
     <row r="2557" ht="15.75" customHeight="1">
-      <c r="A2557" s="2">
-        <v>31.54833333333333</v>
-      </c>
-      <c r="B2557" s="3">
-        <v>378.3842468261719</v>
-      </c>
+      <c r="A2557" s="2"/>
+      <c r="B2557" s="3"/>
     </row>
     <row r="2558" ht="15.75" customHeight="1">
-      <c r="A2558" s="2">
-        <v>31.55833333333333</v>
-      </c>
-      <c r="B2558" s="3">
-        <v>377.5858459472656</v>
-      </c>
+      <c r="A2558" s="2"/>
+      <c r="B2558" s="3"/>
     </row>
     <row r="2559" ht="15.75" customHeight="1">
-      <c r="A2559" s="2">
-        <v>31.56833333333334</v>
-      </c>
-      <c r="B2559" s="3">
-        <v>365.413818359375</v>
-      </c>
+      <c r="A2559" s="2"/>
+      <c r="B2559" s="3"/>
     </row>
     <row r="2560" ht="15.75" customHeight="1">
-      <c r="A2560" s="2">
-        <v>31.57833333333333</v>
-      </c>
-      <c r="B2560" s="3">
-        <v>347.4085693359375</v>
-      </c>
+      <c r="A2560" s="2"/>
+      <c r="B2560" s="3"/>
     </row>
     <row r="2561" ht="15.75" customHeight="1">
-      <c r="A2561" s="2">
-        <v>31.58833333333333</v>
-      </c>
-      <c r="B2561" s="3">
-        <v>348.8135681152344</v>
-      </c>
+      <c r="A2561" s="2"/>
+      <c r="B2561" s="3"/>
     </row>
     <row r="2562" ht="15.75" customHeight="1">
-      <c r="A2562" s="2">
-        <v>31.59833333333334</v>
-      </c>
-      <c r="B2562" s="3">
-        <v>348.3721313476562</v>
-      </c>
+      <c r="A2562" s="2"/>
+      <c r="B2562" s="3"/>
     </row>
     <row r="2563" ht="15.75" customHeight="1">
-      <c r="A2563" s="2">
-        <v>31.59833333333334</v>
-      </c>
+      <c r="A2563" s="2"/>
     </row>
     <row r="2564" ht="15.75" customHeight="1">
-      <c r="A2564" s="2">
-        <v>31.60833333333333</v>
-      </c>
-      <c r="B2564" s="3">
-        <v>73.2066879272461</v>
-      </c>
+      <c r="A2564" s="2"/>
+      <c r="B2564" s="3"/>
     </row>
     <row r="2565" ht="15.75" customHeight="1">
-      <c r="A2565" s="2">
-        <v>31.61833333333333</v>
-      </c>
-      <c r="B2565" s="3">
-        <v>72.73128509521484</v>
-      </c>
+      <c r="A2565" s="2"/>
+      <c r="B2565" s="3"/>
     </row>
     <row r="2566" ht="15.75" customHeight="1">
-      <c r="A2566" s="2">
-        <v>31.62833333333333</v>
-      </c>
-      <c r="B2566" s="3">
-        <v>72.36116027832031</v>
-      </c>
+      <c r="A2566" s="2"/>
+      <c r="B2566" s="3"/>
     </row>
     <row r="2567" ht="15.75" customHeight="1">
-      <c r="A2567" s="2">
-        <v>31.63833333333334</v>
-      </c>
-      <c r="B2567" s="3">
-        <v>72.62081909179688</v>
-      </c>
+      <c r="A2567" s="2"/>
+      <c r="B2567" s="3"/>
     </row>
     <row r="2568" ht="15.75" customHeight="1">
-      <c r="A2568" s="2">
-        <v>31.63833333333334</v>
-      </c>
+      <c r="A2568" s="2"/>
     </row>
     <row r="2569" ht="15.75" customHeight="1">
-      <c r="A2569" s="2">
-        <v>31.64833333333333</v>
-      </c>
-      <c r="B2569" s="3">
-        <v>293.6399230957031</v>
-      </c>
+      <c r="A2569" s="2"/>
+      <c r="B2569" s="3"/>
     </row>
     <row r="2570" ht="15.75" customHeight="1">
-      <c r="A2570" s="2">
-        <v>31.65833333333333</v>
-      </c>
-      <c r="B2570" s="3">
-        <v>289.4961547851562</v>
-      </c>
+      <c r="A2570" s="2"/>
+      <c r="B2570" s="3"/>
     </row>
     <row r="2571" ht="15.75" customHeight="1">
-      <c r="A2571" s="2">
-        <v>31.66833333333334</v>
-      </c>
-      <c r="B2571" s="3">
-        <v>287.1095275878906</v>
-      </c>
+      <c r="A2571" s="2"/>
+      <c r="B2571" s="3"/>
     </row>
     <row r="2572" ht="15.75" customHeight="1">
-      <c r="A2572" s="2">
-        <v>31.67833333333333</v>
-      </c>
-      <c r="B2572" s="3">
-        <v>285.8216552734375</v>
-      </c>
+      <c r="A2572" s="2"/>
+      <c r="B2572" s="3"/>
     </row>
     <row r="2573" ht="15.75" customHeight="1">
-      <c r="A2573" s="2">
-        <v>31.68833333333333</v>
-      </c>
-      <c r="B2573" s="3">
-        <v>284.7236633300781</v>
-      </c>
+      <c r="A2573" s="2"/>
+      <c r="B2573" s="3"/>
     </row>
     <row r="2574" ht="15.75" customHeight="1">
-      <c r="A2574" s="2">
-        <v>31.69833333333333</v>
-      </c>
-      <c r="B2574" s="3">
-        <v>286.9701843261719</v>
-      </c>
+      <c r="A2574" s="2"/>
+      <c r="B2574" s="3"/>
     </row>
     <row r="2575" ht="15.75" customHeight="1">
-      <c r="A2575" s="2">
-        <v>31.69833333333333</v>
-      </c>
+      <c r="A2575" s="2"/>
     </row>
     <row r="2576" ht="15.75" customHeight="1">
-      <c r="A2576" s="2">
-        <v>31.70833333333334</v>
-      </c>
-      <c r="B2576" s="3">
-        <v>93.93759155273438</v>
-      </c>
+      <c r="A2576" s="2"/>
+      <c r="B2576" s="3"/>
     </row>
     <row r="2577" ht="15.75" customHeight="1">
-      <c r="A2577" s="2">
-        <v>31.71833333333333</v>
-      </c>
-      <c r="B2577" s="3">
-        <v>86.6379165649414</v>
-      </c>
+      <c r="A2577" s="2"/>
+      <c r="B2577" s="3"/>
     </row>
     <row r="2578" ht="15.75" customHeight="1">
-      <c r="A2578" s="2">
-        <v>31.72833333333334</v>
-      </c>
+      <c r="A2578" s="2"/>
     </row>
     <row r="2579" ht="15.75" customHeight="1">
-      <c r="A2579" s="2">
-        <v>31.73833333333334</v>
-      </c>
-      <c r="B2579" s="3">
-        <v>71.6734390258789</v>
-      </c>
+      <c r="A2579" s="2"/>
+      <c r="B2579" s="3"/>
     </row>
     <row r="2580" ht="15.75" customHeight="1">
-      <c r="A2580" s="2">
-        <v>31.74833333333333</v>
-      </c>
-      <c r="B2580" s="3">
-        <v>71.59931182861328</v>
-      </c>
+      <c r="A2580" s="2"/>
+      <c r="B2580" s="3"/>
     </row>
     <row r="2581" ht="15.75" customHeight="1">
-      <c r="A2581" s="2">
-        <v>31.75833333333333</v>
-      </c>
-      <c r="B2581" s="3">
-        <v>70.58634185791016</v>
-      </c>
+      <c r="A2581" s="2"/>
+      <c r="B2581" s="3"/>
     </row>
     <row r="2582" ht="15.75" customHeight="1">
-      <c r="A2582" s="2">
-        <v>31.76833333333333</v>
-      </c>
-      <c r="B2582" s="3">
-        <v>88.76506042480469</v>
-      </c>
+      <c r="A2582" s="2"/>
+      <c r="B2582" s="3"/>
     </row>
     <row r="2583" ht="15.75" customHeight="1">
-      <c r="A2583" s="2">
-        <v>31.77833333333334</v>
-      </c>
-      <c r="B2583" s="3">
-        <v>88.03053283691406</v>
-      </c>
+      <c r="A2583" s="2"/>
+      <c r="B2583" s="3"/>
     </row>
     <row r="2584" ht="15.75" customHeight="1">
-      <c r="A2584" s="2">
-        <v>31.77833333333334</v>
-      </c>
+      <c r="A2584" s="2"/>
     </row>
     <row r="2585" ht="15.75" customHeight="1">
-      <c r="A2585" s="2">
-        <v>31.78833333333333</v>
-      </c>
-      <c r="B2585" s="3">
-        <v>175.3336181640625</v>
-      </c>
+      <c r="A2585" s="2"/>
+      <c r="B2585" s="3"/>
     </row>
     <row r="2586" ht="15.75" customHeight="1">
-      <c r="A2586" s="2">
-        <v>31.79833333333333</v>
-      </c>
-      <c r="B2586" s="3">
-        <v>174.4110717773438</v>
-      </c>
+      <c r="A2586" s="2"/>
+      <c r="B2586" s="3"/>
     </row>
     <row r="2587" ht="15.75" customHeight="1">
-      <c r="A2587" s="2">
-        <v>31.80833333333334</v>
-      </c>
-      <c r="B2587" s="3">
-        <v>172.2591552734375</v>
-      </c>
+      <c r="A2587" s="2"/>
+      <c r="B2587" s="3"/>
     </row>
     <row r="2588" ht="15.75" customHeight="1">
-      <c r="A2588" s="2">
-        <v>31.81833333333334</v>
-      </c>
-      <c r="B2588" s="3">
-        <v>171.3900451660156</v>
-      </c>
+      <c r="A2588" s="2"/>
+      <c r="B2588" s="3"/>
     </row>
     <row r="2589" ht="15.75" customHeight="1">
-      <c r="A2589" s="2">
-        <v>31.82833333333333</v>
-      </c>
-      <c r="B2589" s="3">
-        <v>171.5803680419922</v>
-      </c>
+      <c r="A2589" s="2"/>
+      <c r="B2589" s="3"/>
     </row>
     <row r="2590" ht="15.75" customHeight="1">
-      <c r="A2590" s="2">
-        <v>31.83833333333333</v>
-      </c>
-      <c r="B2590" s="3">
-        <v>163.9794006347656</v>
-      </c>
+      <c r="A2590" s="2"/>
+      <c r="B2590" s="3"/>
     </row>
     <row r="2591" ht="15.75" customHeight="1">
-      <c r="A2591" s="2">
-        <v>31.84833333333334</v>
-      </c>
-      <c r="B2591" s="3">
-        <v>164.6298522949219</v>
-      </c>
+      <c r="A2591" s="2"/>
+      <c r="B2591" s="3"/>
     </row>
     <row r="2592" ht="15.75" customHeight="1">
-      <c r="A2592" s="2">
-        <v>31.85833333333333</v>
-      </c>
-      <c r="B2592" s="3">
-        <v>165.1906433105469</v>
-      </c>
+      <c r="A2592" s="2"/>
+      <c r="B2592" s="3"/>
     </row>
     <row r="2593" ht="15.75" customHeight="1">
-      <c r="A2593" s="2">
-        <v>31.86833333333333</v>
-      </c>
-      <c r="B2593" s="3">
-        <v>167.0840301513672</v>
-      </c>
+      <c r="A2593" s="2"/>
+      <c r="B2593" s="3"/>
     </row>
     <row r="2594" ht="15.75" customHeight="1">
-      <c r="A2594" s="2">
-        <v>31.87833333333333</v>
-      </c>
-      <c r="B2594" s="3">
-        <v>167.5724945068359</v>
-      </c>
+      <c r="A2594" s="2"/>
+      <c r="B2594" s="3"/>
     </row>
     <row r="2595" ht="15.75" customHeight="1">
-      <c r="A2595" s="2">
-        <v>31.88833333333334</v>
-      </c>
-      <c r="B2595" s="3">
-        <v>168.0228118896484</v>
-      </c>
+      <c r="A2595" s="2"/>
+      <c r="B2595" s="3"/>
     </row>
     <row r="2596" ht="15.75" customHeight="1">
-      <c r="A2596" s="2">
-        <v>31.89833333333333</v>
-      </c>
-      <c r="B2596" s="3">
-        <v>168.4118957519531</v>
-      </c>
+      <c r="A2596" s="2"/>
+      <c r="B2596" s="3"/>
     </row>
     <row r="2597" ht="15.75" customHeight="1">
-      <c r="A2597" s="2">
-        <v>31.89833333333333</v>
-      </c>
+      <c r="A2597" s="2"/>
     </row>
     <row r="2598" ht="15.75" customHeight="1">
-      <c r="A2598" s="2">
-        <v>31.90833333333333</v>
-      </c>
-      <c r="B2598" s="3">
-        <v>84.20744323730469</v>
-      </c>
+      <c r="A2598" s="2"/>
+      <c r="B2598" s="3"/>
     </row>
     <row r="2599" ht="15.75" customHeight="1">
-      <c r="A2599" s="2">
-        <v>31.91833333333334</v>
-      </c>
-      <c r="B2599" s="3">
-        <v>83.7066421508789</v>
-      </c>
+      <c r="A2599" s="2"/>
+      <c r="B2599" s="3"/>
     </row>
     <row r="2600" ht="15.75" customHeight="1">
-      <c r="A2600" s="2">
-        <v>31.92833333333333</v>
-      </c>
-      <c r="B2600" s="3">
-        <v>104.5489044189453</v>
-      </c>
+      <c r="A2600" s="2"/>
+      <c r="B2600" s="3"/>
     </row>
     <row r="2601" ht="15.75" customHeight="1">
-      <c r="A2601" s="2">
-        <v>31.93833333333333</v>
-      </c>
-      <c r="B2601" s="3">
-        <v>67.78349304199219</v>
-      </c>
+      <c r="A2601" s="2"/>
+      <c r="B2601" s="3"/>
     </row>
     <row r="2602" ht="15.75" customHeight="1">
-      <c r="A2602" s="2">
-        <v>31.93833333333333</v>
-      </c>
+      <c r="A2602" s="2"/>
     </row>
     <row r="2603" ht="15.75" customHeight="1">
-      <c r="A2603" s="2">
-        <v>31.94833333333333</v>
-      </c>
-      <c r="B2603" s="3">
-        <v>197.5421142578125</v>
-      </c>
+      <c r="A2603" s="2"/>
+      <c r="B2603" s="3"/>
     </row>
     <row r="2604" ht="15.75" customHeight="1">
-      <c r="A2604" s="2">
-        <v>31.95833333333334</v>
-      </c>
-      <c r="B2604" s="3">
-        <v>198.4172515869141</v>
-      </c>
+      <c r="A2604" s="2"/>
+      <c r="B2604" s="3"/>
     </row>
     <row r="2605" ht="15.75" customHeight="1">
-      <c r="A2605" s="2">
-        <v>31.96833333333333</v>
-      </c>
-      <c r="B2605" s="3">
-        <v>197.4205780029297</v>
-      </c>
+      <c r="A2605" s="2"/>
+      <c r="B2605" s="3"/>
     </row>
     <row r="2606" ht="15.75" customHeight="1">
-      <c r="A2606" s="2">
-        <v>31.97833333333334</v>
-      </c>
-      <c r="B2606" s="3">
-        <v>197.4684600830078</v>
-      </c>
+      <c r="A2606" s="2"/>
+      <c r="B2606" s="3"/>
     </row>
     <row r="2607" ht="15.75" customHeight="1">
-      <c r="A2607" s="2">
-        <v>31.98833333333334</v>
-      </c>
-      <c r="B2607" s="3">
-        <v>188.4786224365234</v>
-      </c>
+      <c r="A2607" s="2"/>
+      <c r="B2607" s="3"/>
     </row>
     <row r="2608" ht="15.75" customHeight="1">
-      <c r="A2608" s="2">
-        <v>31.99833333333333</v>
-      </c>
-      <c r="B2608" s="3">
-        <v>187.9543151855469</v>
-      </c>
+      <c r="A2608" s="2"/>
+      <c r="B2608" s="3"/>
     </row>
     <row r="2609" ht="15.75" customHeight="1">
-      <c r="A2609" s="2">
-        <v>32.00833333333333</v>
-      </c>
-      <c r="B2609" s="3">
-        <v>178.4929809570312</v>
-      </c>
+      <c r="A2609" s="2"/>
+      <c r="B2609" s="3"/>
     </row>
     <row r="2610" ht="15.75" customHeight="1">
-      <c r="A2610" s="2">
-        <v>32.01833333333333</v>
-      </c>
-      <c r="B2610" s="3">
-        <v>178.6670684814453</v>
-      </c>
+      <c r="A2610" s="2"/>
+      <c r="B2610" s="3"/>
     </row>
     <row r="2611" ht="15.75" customHeight="1">
-      <c r="A2611" s="2">
-        <v>32.02833333333334</v>
-      </c>
-      <c r="B2611" s="3">
-        <v>187.40771484375</v>
-      </c>
+      <c r="A2611" s="2"/>
+      <c r="B2611" s="3"/>
     </row>
     <row r="2612" ht="15.75" customHeight="1">
-      <c r="A2612" s="2">
-        <v>32.14833333333333</v>
-      </c>
+      <c r="A2612" s="2"/>
     </row>
     <row r="2613" ht="15.75" customHeight="1">
-      <c r="A2613" s="2">
-        <v>32.15833333333333</v>
-      </c>
-      <c r="B2613" s="3">
-        <v>183.7842102050781</v>
-      </c>
+      <c r="A2613" s="2"/>
+      <c r="B2613" s="3"/>
     </row>
     <row r="2614" ht="15.75" customHeight="1">
-      <c r="A2614" s="2">
-        <v>32.16833333333334</v>
-      </c>
-      <c r="B2614" s="3">
-        <v>177.712646484375</v>
-      </c>
+      <c r="A2614" s="2"/>
+      <c r="B2614" s="3"/>
     </row>
     <row r="2615" ht="15.75" customHeight="1">
-      <c r="A2615" s="2">
-        <v>32.17833333333333</v>
-      </c>
-      <c r="B2615" s="3">
-        <v>175.6324920654297</v>
-      </c>
+      <c r="A2615" s="2"/>
+      <c r="B2615" s="3"/>
     </row>
     <row r="2616" ht="15.75" customHeight="1">
-      <c r="A2616" s="2">
-        <v>32.18833333333333</v>
-      </c>
-      <c r="B2616" s="3">
-        <v>172.2797698974609</v>
-      </c>
+      <c r="A2616" s="2"/>
+      <c r="B2616" s="3"/>
     </row>
     <row r="2617" ht="15.75" customHeight="1">
-      <c r="A2617" s="2">
-        <v>32.19833333333334</v>
-      </c>
-      <c r="B2617" s="3">
-        <v>168.7670745849609</v>
-      </c>
+      <c r="A2617" s="2"/>
+      <c r="B2617" s="3"/>
     </row>
     <row r="2618" ht="15.75" customHeight="1">
-      <c r="A2618" s="2">
-        <v>32.20833333333334</v>
-      </c>
-      <c r="B2618" s="3">
-        <v>168.0787200927734</v>
-      </c>
+      <c r="A2618" s="2"/>
+      <c r="B2618" s="3"/>
     </row>
     <row r="2619" ht="15.75" customHeight="1">
-      <c r="A2619" s="2">
-        <v>32.21833333333333</v>
-      </c>
-      <c r="B2619" s="3">
-        <v>167.6222381591797</v>
-      </c>
+      <c r="A2619" s="2"/>
+      <c r="B2619" s="3"/>
     </row>
     <row r="2620" ht="15.75" customHeight="1">
-      <c r="A2620" s="2">
-        <v>32.22833333333334</v>
-      </c>
-      <c r="B2620" s="3">
-        <v>167.9656524658203</v>
-      </c>
+      <c r="A2620" s="2"/>
+      <c r="B2620" s="3"/>
     </row>
     <row r="2621" ht="15.75" customHeight="1">
-      <c r="A2621" s="2">
-        <v>32.23833333333333</v>
-      </c>
-      <c r="B2621" s="3">
-        <v>168.5245361328125</v>
-      </c>
+      <c r="A2621" s="2"/>
+      <c r="B2621" s="3"/>
     </row>
     <row r="2622" ht="15.75" customHeight="1">
-      <c r="A2622" s="2">
-        <v>32.24833333333333</v>
-      </c>
-      <c r="B2622" s="3">
-        <v>169.4394989013672</v>
-      </c>
+      <c r="A2622" s="2"/>
+      <c r="B2622" s="3"/>
     </row>
     <row r="2623" ht="15.75" customHeight="1">
-      <c r="A2623" s="2">
-        <v>32.25833333333333</v>
-      </c>
-      <c r="B2623" s="3">
-        <v>170.3506927490234</v>
-      </c>
+      <c r="A2623" s="2"/>
+      <c r="B2623" s="3"/>
     </row>
     <row r="2624" ht="15.75" customHeight="1">
-      <c r="A2624" s="2">
-        <v>32.26833333333333</v>
-      </c>
-      <c r="B2624" s="3">
-        <v>170.4350738525391</v>
-      </c>
+      <c r="A2624" s="2"/>
+      <c r="B2624" s="3"/>
     </row>
     <row r="2625" ht="15.75" customHeight="1">
-      <c r="A2625" s="2">
-        <v>32.27833333333334</v>
-      </c>
-      <c r="B2625" s="3">
-        <v>172.0368804931641</v>
-      </c>
+      <c r="A2625" s="2"/>
+      <c r="B2625" s="3"/>
     </row>
     <row r="2626" ht="15.75" customHeight="1">
-      <c r="A2626" s="2">
-        <v>32.28833333333333</v>
-      </c>
-      <c r="B2626" s="3">
-        <v>170.3018341064453</v>
-      </c>
+      <c r="A2626" s="2"/>
+      <c r="B2626" s="3"/>
     </row>
     <row r="2627" ht="15.75" customHeight="1">
-      <c r="A2627" s="2">
-        <v>32.29833333333333</v>
-      </c>
-      <c r="B2627" s="3">
-        <v>170.2083587646484</v>
-      </c>
+      <c r="A2627" s="2"/>
+      <c r="B2627" s="3"/>
     </row>
     <row r="2628" ht="15.75" customHeight="1">
-      <c r="A2628" s="2">
-        <v>32.30833333333334</v>
-      </c>
-      <c r="B2628" s="3">
-        <v>168.4323883056641</v>
-      </c>
+      <c r="A2628" s="2"/>
+      <c r="B2628" s="3"/>
     </row>
     <row r="2629" ht="15.75" customHeight="1">
-      <c r="A2629" s="2">
-        <v>32.31833333333334</v>
-      </c>
+      <c r="A2629" s="2"/>
     </row>
     <row r="2630" ht="15.75" customHeight="1">
-      <c r="A2630" s="2">
-        <v>32.32833333333333</v>
-      </c>
-      <c r="B2630" s="3">
-        <v>163.1427612304688</v>
-      </c>
+      <c r="A2630" s="2"/>
+      <c r="B2630" s="3"/>
     </row>
     <row r="2631" ht="15.75" customHeight="1">
-      <c r="A2631" s="2">
-        <v>32.33833333333334</v>
-      </c>
-      <c r="B2631" s="3">
-        <v>156.6971130371094</v>
-      </c>
+      <c r="A2631" s="2"/>
+      <c r="B2631" s="3"/>
     </row>
     <row r="2632" ht="15.75" customHeight="1">
-      <c r="A2632" s="2">
-        <v>32.34833333333333</v>
-      </c>
-      <c r="B2632" s="3">
-        <v>155.4387969970703</v>
-      </c>
+      <c r="A2632" s="2"/>
+      <c r="B2632" s="3"/>
     </row>
     <row r="2633" ht="15.75" customHeight="1">
-      <c r="A2633" s="2">
-        <v>32.35833333333333</v>
-      </c>
-      <c r="B2633" s="3">
-        <v>154.7712249755859</v>
-      </c>
+      <c r="A2633" s="2"/>
+      <c r="B2633" s="3"/>
     </row>
     <row r="2634" ht="15.75" customHeight="1">
-      <c r="A2634" s="2">
-        <v>32.36833333333334</v>
-      </c>
-      <c r="B2634" s="3">
-        <v>153.6117401123047</v>
-      </c>
+      <c r="A2634" s="2"/>
+      <c r="B2634" s="3"/>
     </row>
     <row r="2635" ht="15.75" customHeight="1">
-      <c r="A2635" s="2">
-        <v>32.37833333333333</v>
-      </c>
-      <c r="B2635" s="3">
-        <v>150.6729736328125</v>
-      </c>
+      <c r="A2635" s="2"/>
+      <c r="B2635" s="3"/>
     </row>
     <row r="2636" ht="15.75" customHeight="1">
-      <c r="A2636" s="2">
-        <v>32.38833333333334</v>
-      </c>
-      <c r="B2636" s="3">
-        <v>149.7633361816406</v>
-      </c>
+      <c r="A2636" s="2"/>
+      <c r="B2636" s="3"/>
     </row>
     <row r="2637" ht="15.75" customHeight="1">
-      <c r="A2637" s="2">
-        <v>32.39833333333333</v>
-      </c>
-      <c r="B2637" s="3">
-        <v>150.2164764404297</v>
-      </c>
+      <c r="A2637" s="2"/>
+      <c r="B2637" s="3"/>
     </row>
   </sheetData>
   <printOptions/>

</xml_diff>